<commit_message>
amélioration du programme de rapprochement avec ajout de la page d'authentification
</commit_message>
<xml_diff>
--- a/documents/relevé.xlsx
+++ b/documents/relevé.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G57"/>
+  <dimension ref="A1:G94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,12 +471,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>06/10/2025</t>
+          <t>03/11/2025</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>06/10/2025</t>
+          <t>03/11/2025</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -491,7 +491,7 @@
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>18960597</v>
+        <v>324155423</v>
       </c>
     </row>
     <row r="3">
@@ -500,27 +500,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>06/10/2025</t>
+          <t>03/11/2025</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>06/10/2025</t>
+          <t>03/11/2025</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000763 Ret cheq N 6000763 du 06/10/2025 Porteur : AYISSOU ELOM KOFFI 91551295</t>
+          <t>ESPECE CPT COURANT especes Bord N 223496 BELARO 90915582</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>767000</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>534880</v>
       </c>
       <c r="G3" t="n">
-        <v>18193597</v>
+        <v>324690303</v>
       </c>
     </row>
     <row r="4">
@@ -529,27 +529,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>06/10/2025</t>
+          <t>03/11/2025</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>06/10/2025</t>
+          <t>03/11/2025</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000760 Ret cheq N 6000760 du 06/10/2025 Porteur : BADAKI ABLO MNI-B 91332293</t>
+          <t>ESPECE CPT COURANT especes Bord N 903251 T LUCIE92332829</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>1249000</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>2271300</v>
       </c>
       <c r="G4" t="n">
-        <v>16944597</v>
+        <v>326961603</v>
       </c>
     </row>
     <row r="5">
@@ -558,27 +558,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>06/10/2025</t>
+          <t>03/11/2025</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>06/10/2025</t>
+          <t>03/11/2025</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000761 Ret cheq N 6000761 du 06/10/2025 Porteur : PORO K EDJAREGUEW</t>
+          <t>ESPECE CPT COURANT especes Bord N 903253 T LUCIE 92332829</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>562800</v>
+        <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>107775</v>
       </c>
       <c r="G5" t="n">
-        <v>16381797</v>
+        <v>327069378</v>
       </c>
     </row>
     <row r="6">
@@ -587,27 +587,27 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>07/10/2025</t>
+          <t>03/11/2025</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>07/10/2025</t>
+          <t>05/11/2025</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000762 Ret cheq N 6000762 du 07/10/2025 Porteur : WOROU KODJO DODUJI</t>
+          <t>CHEQ SBF AUTRE BANQ SP SBF 5508165</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>574000</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>2544800</v>
       </c>
       <c r="G6" t="n">
-        <v>15807797</v>
+        <v>329614178</v>
       </c>
     </row>
     <row r="7">
@@ -616,27 +616,27 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>08/10/2025</t>
+          <t>03/11/2025</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>08/10/2025</t>
+          <t>05/11/2025</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000765 Ret cheq N 6000765 du 08/10/2025 Porteur : TABATA KOUMSOGA 90936649</t>
+          <t>CHEQ SBF AUTRE BANQ SP SBF 2072863</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>608000</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>646000</v>
       </c>
       <c r="G7" t="n">
-        <v>15199797</v>
+        <v>330260178</v>
       </c>
     </row>
     <row r="8">
@@ -645,27 +645,27 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>08/10/2025</t>
+          <t>03/11/2025</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>08/10/2025</t>
+          <t>31/10/2025</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000756 Ret cheq N 6000756 du 08/10/2025 Porteur : MAWUSSI KOFFI</t>
+          <t>NOS CAISSES fav. CODIP (COMPAGNIE DE DISTRIBUTION 154434 - 01101 - VIRT</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>216000</v>
+        <v>89500</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>14983797</v>
+        <v>330170678</v>
       </c>
     </row>
     <row r="9">
@@ -674,27 +674,27 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>09/10/2025</t>
+          <t>04/11/2025</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>09/10/2025</t>
+          <t>04/11/2025</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000766 Ret cheq N 6000766 du 09/10/2025 Porteur : DOLOU, ESSOLAKINA 90242454</t>
+          <t>ESPECE CPT COURANT especes Bord N 903599 T LUCIE 92332829</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>650300</v>
+        <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>2555800</v>
       </c>
       <c r="G9" t="n">
-        <v>14333497</v>
+        <v>332726478</v>
       </c>
     </row>
     <row r="10">
@@ -703,27 +703,27 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>09/10/2025</t>
+          <t>04/11/2025</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>08/10/2025</t>
+          <t>03/11/2025</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>CHEQUE RETOUR DE COMPENSATION Chq OTG n 6000769</t>
+          <t>RETOUR DE COMPENSATION OTG n 5810872</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>320000</v>
+        <v>1384740</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>14013497</v>
+        <v>331341738</v>
       </c>
     </row>
     <row r="11">
@@ -732,27 +732,27 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>13/10/2025</t>
+          <t>04/11/2025</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>13/10/2025</t>
+          <t>03/11/2025</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000767 Ret cheq N 6000767 du 13/10/2025 Porteur : BAWILISSIM DONSOSSOU 90021198</t>
+          <t>RETOUR DE COMPENSATION OTG n 5810871</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>541000</v>
+        <v>1852000</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>13472497</v>
+        <v>329489738</v>
       </c>
     </row>
     <row r="12">
@@ -761,27 +761,27 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>13/10/2025</t>
+          <t>04/11/2025</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>13/10/2025</t>
+          <t>03/11/2025</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000768 Ret cheq N 6000768 du 13/10/2025 Porteur : LAMBONI SIELPAK</t>
+          <t>RETOUR DE COMPENSATION OTG n 5810873</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>200000</v>
+        <v>1400000</v>
       </c>
       <c r="F12" t="n">
         <v>0</v>
       </c>
       <c r="G12" t="n">
-        <v>13272497</v>
+        <v>328089738</v>
       </c>
     </row>
     <row r="13">
@@ -790,27 +790,27 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>23/10/2025</t>
+          <t>05/11/2025</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>23/10/2025</t>
+          <t>05/11/2025</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>VERSEMENT ESPECE CPT COURANT Versement especes Bord N 900516 ATTIGLOH KOFFI M 93174711</t>
+          <t>ESPECE CPT COURANT especes Bord N 904049 T LUCIE 92332829</t>
         </is>
       </c>
       <c r="E13" t="n">
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>1400</v>
+        <v>2478675</v>
       </c>
       <c r="G13" t="n">
-        <v>13273897</v>
+        <v>330568413</v>
       </c>
     </row>
     <row r="14">
@@ -819,27 +819,27 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10/11/2025</t>
+          <t>06/11/2025</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>10/11/2025</t>
+          <t>06/11/2025</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000652 Ret cheq N 6000652 du 10/11/2025 Porteur : MOUSSA GANIOU 90033563</t>
+          <t>ESPECES CPT 5689824</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>277000</v>
+        <v>5000000</v>
       </c>
       <c r="F14" t="n">
         <v>0</v>
       </c>
       <c r="G14" t="n">
-        <v>12996897</v>
+        <v>325568413</v>
       </c>
     </row>
     <row r="15">
@@ -848,27 +848,27 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10/11/2025</t>
+          <t>06/11/2025</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>10/11/2025</t>
+          <t>06/11/2025</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000772 Ret cheq N 6000772 du 10/11/2025 - MAKO ESSOFA 90362152 Porteur : MAKO ESSOFA 90362152</t>
+          <t>ESPECE CPT COURANT especes Bord N 904451 K EDEM 90978863</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>230000</v>
+        <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>3298850</v>
       </c>
       <c r="G15" t="n">
-        <v>12766897</v>
+        <v>328867263</v>
       </c>
     </row>
     <row r="16">
@@ -877,27 +877,27 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>10/11/2025</t>
+          <t>06/11/2025</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>10/11/2025</t>
+          <t>05/11/2025</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000779 Ret cheq N 6000779 du 10/11/2025 Porteur : TEKO MENSAH 90152664</t>
+          <t>RETOUR DE COMPENSATION OTG n 5810865</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>350000</v>
+        <v>3760721</v>
       </c>
       <c r="F16" t="n">
         <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>12416897</v>
+        <v>325106542</v>
       </c>
     </row>
     <row r="17">
@@ -906,27 +906,27 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>10/11/2025</t>
+          <t>06/11/2025</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>10/11/2025</t>
+          <t>05/11/2025</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000781 Ret cheq N 6000781 du 10/11/2025 Porteur : KAMOKI MAWABA 91571987</t>
+          <t>RETOUR DE COMPENSATION OTG n 5810878</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>259000</v>
+        <v>545000</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>12157897</v>
+        <v>324561542</v>
       </c>
     </row>
     <row r="18">
@@ -935,27 +935,27 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>10/11/2025</t>
+          <t>06/11/2025</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>10/11/2025</t>
+          <t>05/11/2025</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000780 Ret cheq N 6000780 du 10/11/2025 Porteur : ASSONDE K DITORGUE 93070886</t>
+          <t>AUTRES AGENCES fav. ETS GLOBALS SERVICES GROUP TOGO 160143 - 01101 - BR 25000280</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>350000</v>
+        <v>390000</v>
       </c>
       <c r="F18" t="n">
         <v>0</v>
       </c>
       <c r="G18" t="n">
-        <v>11807897</v>
+        <v>324171542</v>
       </c>
     </row>
     <row r="19">
@@ -964,27 +964,27 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>10/11/2025</t>
+          <t>07/11/2025</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>10/11/2025</t>
+          <t>07/11/2025</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000656 Ret cheq N 6000656 du 10/11/2025 Porteur : AMEGBOR KOFFI 90125043</t>
+          <t>ESPECES CPT 5689823 N 5689823 : ANENYA KOMIVI EDEM 90978863</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>280000</v>
+        <v>90000</v>
       </c>
       <c r="F19" t="n">
         <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>11527897</v>
+        <v>324081542</v>
       </c>
     </row>
     <row r="20">
@@ -993,27 +993,27 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11/11/2025</t>
+          <t>07/11/2025</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>11/11/2025</t>
+          <t>07/11/2025</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000657 Ret cheq N 6000657 du 11/11/2025 Porteur : BLEWOU COMLAN YOM</t>
+          <t>ESPECE CPT COURANT especes Bord N 904897 K EDEM 90978863</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>280000</v>
+        <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>0</v>
+        <v>2506725</v>
       </c>
       <c r="G20" t="n">
-        <v>11247897</v>
+        <v>326588267</v>
       </c>
     </row>
     <row r="21">
@@ -1022,27 +1022,27 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>11/11/2025</t>
+          <t>07/11/2025</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>11/11/2025</t>
+          <t>06/11/2025</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000777 Ret cheq N 6000777 du 11/11/2025 Porteur : BADAKI ABALO M B 91332293</t>
+          <t>RETOUR DE COMPENSATION OTG n 5810879</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>349000</v>
+        <v>4332477</v>
       </c>
       <c r="F21" t="n">
         <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>10898897</v>
+        <v>322255790</v>
       </c>
     </row>
     <row r="22">
@@ -1051,27 +1051,27 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
+          <t>07/11/2025</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
           <t>11/11/2025</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>11/11/2025</t>
-        </is>
-      </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000667 Ret cheq N 6000667 du 11/11/2025 - MONTANT MINYO EGA 92101033 Porteur : MONTANT MINYO EGA 92101033</t>
+          <t>CHEQUES AUTRE BANQUE 1818147 - CORIS BANK TOGO BANK TOGO</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>136000</v>
+        <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>0</v>
+        <v>244500</v>
       </c>
       <c r="G22" t="n">
-        <v>10762897</v>
+        <v>322500290</v>
       </c>
     </row>
     <row r="23">
@@ -1080,27 +1080,27 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>12/11/2025</t>
+          <t>07/11/2025</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>12/11/2025</t>
+          <t>10/11/2025</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000655 Ret cheq N 6000655 du 12/11/2025 Porteur : ATTIGLOH KOFFI MAWULI 93174711</t>
+          <t>NOS CAISSES ord. C.H.U SYLVANUS OLYMPIO - 01101 - DIV FACTS</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>76000</v>
+        <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>0</v>
+        <v>1093350</v>
       </c>
       <c r="G23" t="n">
-        <v>10686897</v>
+        <v>323593640</v>
       </c>
     </row>
     <row r="24">
@@ -1109,27 +1109,27 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>12/11/2025</t>
+          <t>07/11/2025</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>12/11/2025</t>
+          <t>10/11/2025</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000654 Ret cheq N 6000654 du 12/11/2025 Porteur : LOAGUI YOUMANE 90224409</t>
+          <t>RECU COMPENSATION ord. G C A SINISTRE 1 BANKSIEGEOCT2025 PREST 4</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>182000</v>
+        <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>0</v>
+        <v>15800</v>
       </c>
       <c r="G24" t="n">
-        <v>10504897</v>
+        <v>323609440</v>
       </c>
     </row>
     <row r="25">
@@ -1138,27 +1138,27 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>12/11/2025</t>
+          <t>07/11/2025</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>12/11/2025</t>
+          <t>10/11/2025</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000794 Ret cheq N 6000794 du 12/11/2025 Porteur : LAOGUI YOUMANE 90224409</t>
+          <t>RECU COMPENSATION ord. G C A SINISTRE 1 BANKSIEGESEPT2025 PREST</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>139000</v>
+        <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>0</v>
+        <v>36900</v>
       </c>
       <c r="G25" t="n">
-        <v>10365897</v>
+        <v>323646340</v>
       </c>
     </row>
     <row r="26">
@@ -1167,27 +1167,27 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>12/11/2025</t>
+          <t>10/11/2025</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>12/11/2025</t>
+          <t>10/11/2025</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000770 Ret cheq N 6000770 du 12/11/2025 Porteur : TOUGOUMA ESSO-MONDJONNA</t>
+          <t>ESPECE CPT COURANT especes Bord N 905432</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>349000</v>
+        <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>0</v>
+        <v>441985</v>
       </c>
       <c r="G26" t="n">
-        <v>10016897</v>
+        <v>324088325</v>
       </c>
     </row>
     <row r="27">
@@ -1196,27 +1196,27 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>12/11/2025</t>
+          <t>10/11/2025</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>12/11/2025</t>
+          <t>10/11/2025</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000771 Ret cheq N 6000771 du 12/11/2025 Porteur : TCHA-THOM A 91820620</t>
+          <t>ESPECE CPT COURANT especes Bord N 905433 T LUCIE 92332829</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>349000</v>
+        <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>0</v>
+        <v>1697400</v>
       </c>
       <c r="G27" t="n">
-        <v>9667897</v>
+        <v>325785725</v>
       </c>
     </row>
     <row r="28">
@@ -1225,27 +1225,27 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>13/11/2025</t>
+          <t>11/11/2025</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>13/11/2025</t>
+          <t>11/11/2025</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000789 Ret cheq N 6000789 du 13/11/2025</t>
+          <t>ESPECE CPT COURANT especes Bord N 905902 T LUCIE 92332829</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>389500</v>
+        <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>0</v>
+        <v>3220475</v>
       </c>
       <c r="G28" t="n">
-        <v>9278397</v>
+        <v>329006200</v>
       </c>
     </row>
     <row r="29">
@@ -1254,27 +1254,27 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>13/11/2025</t>
+          <t>11/11/2025</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>13/11/2025</t>
+          <t>10/11/2025</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000788 Ret cheq N 6000788 du 13/11/2025 Porteur : KAMASSA KOMLAN 92710436</t>
+          <t>RETOUR DE COMPENSATION OTG n 5810877</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>392500</v>
+        <v>350000</v>
       </c>
       <c r="F29" t="n">
         <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>8885897</v>
+        <v>328656200</v>
       </c>
     </row>
     <row r="30">
@@ -1283,27 +1283,27 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>13/11/2025</t>
+          <t>12/11/2025</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>13/11/2025</t>
+          <t>11/11/2025</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000791 Ret cheq N 6000791 du 13/11/2025 Porteur : ELIASSOU MARIAME 91323671</t>
+          <t>RETOUR DE COMPENSATION OTG n 5810880</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>385000</v>
+        <v>654581</v>
       </c>
       <c r="F30" t="n">
         <v>0</v>
       </c>
       <c r="G30" t="n">
-        <v>8500897</v>
+        <v>328001619</v>
       </c>
     </row>
     <row r="31">
@@ -1312,27 +1312,27 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>13/11/2025</t>
+          <t>12/11/2025</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>13/11/2025</t>
+          <t>11/11/2025</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000784 Ret cheq N 6000784 du 13/11/2025 Porteur : SIZING PYABALO/TCHOTCHO FEGBABE</t>
+          <t>RETOUR DE COMPENSATION OTG n 5810874</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>229000</v>
+        <v>235000</v>
       </c>
       <c r="F31" t="n">
         <v>0</v>
       </c>
       <c r="G31" t="n">
-        <v>8271897</v>
+        <v>327766619</v>
       </c>
     </row>
     <row r="32">
@@ -1341,27 +1341,27 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>14/11/2025</t>
+          <t>13/11/2025</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>14/11/2025</t>
+          <t>13/11/2025</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000799 Ret cheq N 6000799 du 14/11/2025 Porteur : EKOUWONOU KOKOU MAWOUENA</t>
+          <t>ESPECE CPT COURANT especes Bord N 906730 T LUCIE 92332825</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>238500</v>
+        <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>0</v>
+        <v>2859725</v>
       </c>
       <c r="G32" t="n">
-        <v>8033397</v>
+        <v>330626344</v>
       </c>
     </row>
     <row r="33">
@@ -1370,27 +1370,27 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>14/11/2025</t>
+          <t>13/11/2025</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>14/11/2025</t>
+          <t>13/11/2025</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000775 Ret cheq N 6000775 du 14/11/2025 Porteur : WOLOU IFABI</t>
+          <t>ESPECE CPT COURANT especes Bord N 906731 T LUCIE 92332829</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>225000</v>
+        <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>0</v>
+        <v>2380485</v>
       </c>
       <c r="G33" t="n">
-        <v>7808397</v>
+        <v>333006829</v>
       </c>
     </row>
     <row r="34">
@@ -1399,27 +1399,27 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>17/11/2025</t>
+          <t>13/11/2025</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17/11/2025</t>
+          <t>14/11/2025</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000800 Ret cheq N 6000800 du 17/11/2025 Porteur : TCHALON AKPANTO 92 64 62 28</t>
+          <t>CHEQUES SBF INTERNE chq OTG</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>385000</v>
+        <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>0</v>
+        <v>166600</v>
       </c>
       <c r="G34" t="n">
-        <v>7423397</v>
+        <v>333173429</v>
       </c>
     </row>
     <row r="35">
@@ -1428,27 +1428,27 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>17/11/2025</t>
+          <t>14/11/2025</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>17/11/2025</t>
+          <t>14/11/2025</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000651 Ret cheq N 6000651 du 17/11/2025 Porteur : LARE BAKENANME 91 97 60 08</t>
+          <t>ESPECE CPT COURANT especes Bord N 907164 T LUCIE 92332829</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>400000</v>
+        <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>0</v>
+        <v>1889375</v>
       </c>
       <c r="G35" t="n">
-        <v>7023397</v>
+        <v>335062804</v>
       </c>
     </row>
     <row r="36">
@@ -1457,27 +1457,27 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>17/11/2025</t>
+          <t>14/11/2025</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>17/11/2025</t>
+          <t>14/11/2025</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000778 Ret cheq N 6000778 du 17/11/2025 Porteur : LADOUKPO ESSEVI 90547112</t>
+          <t>ESPECE CPT COURANT especes Bord N 907165 T LUCIE 92332829</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>229000</v>
+        <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>0</v>
+        <v>3065405</v>
       </c>
       <c r="G36" t="n">
-        <v>6794397</v>
+        <v>338128209</v>
       </c>
     </row>
     <row r="37">
@@ -1496,17 +1496,17 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000797 Ret cheq N 6000797</t>
+          <t>ESPECE CPT COURANT especes Bord N 224333 BELARO 90915582</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>352500</v>
+        <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>0</v>
+        <v>333530</v>
       </c>
       <c r="G37" t="n">
-        <v>644189747</v>
+        <v>338461739</v>
       </c>
     </row>
     <row r="38">
@@ -1525,17 +1525,17 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000774 Ret cheq N 6000774 du 17/11/2025 Porteur : KATO KOSSI</t>
+          <t>ESPECE CPT COURANT especes Bord N 907996 T LUCIE 92332825</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>390000</v>
+        <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>0</v>
+        <v>1746250</v>
       </c>
       <c r="G38" t="n">
-        <v>6051897</v>
+        <v>340207989</v>
       </c>
     </row>
     <row r="39">
@@ -1549,22 +1549,22 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>14/11/2025</t>
+          <t>17/11/2025</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>REMISE CHEQUES SBF INTERNE Paiemt chq OTG n 6000795 NEVE 160531 - 01014 -</t>
+          <t>ESPECE CPT COURANT especes Bord N 907999</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>139000</v>
+        <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>0</v>
+        <v>420385</v>
       </c>
       <c r="G39" t="n">
-        <v>5912897</v>
+        <v>340628374</v>
       </c>
     </row>
     <row r="40">
@@ -1583,17 +1583,17 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000790 Ret cheq N 6000790 du 18/11/2025 Porteur : SANSANE GNANDI 91276946</t>
+          <t>ESPECE CPT COURANT especes Bord N 216560 79302844</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>77000</v>
+        <v>0</v>
       </c>
       <c r="F40" t="n">
-        <v>0</v>
+        <v>216800</v>
       </c>
       <c r="G40" t="n">
-        <v>5835897</v>
+        <v>340845174</v>
       </c>
     </row>
     <row r="41">
@@ -1612,17 +1612,17 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000783 Ret cheq N 6000783 du 18/11/2025 Porteur : TEKO MINOGBLON 92418428</t>
+          <t>ESPECE CPT COURANT especes Bord N 908304 T LUCIE 92332829</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>322500</v>
+        <v>0</v>
       </c>
       <c r="F41" t="n">
-        <v>0</v>
+        <v>2852800</v>
       </c>
       <c r="G41" t="n">
-        <v>5513397</v>
+        <v>343697974</v>
       </c>
     </row>
     <row r="42">
@@ -1631,27 +1631,27 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>18/11/2025</t>
+          <t>19/11/2025</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>18/11/2025</t>
+          <t>19/11/2025</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000787 Ret cheq N 6000787 du 18/11/2025 Porteur : ATTIGLOH KOFFI MAWULI</t>
+          <t>ESPECE CPT COURANT especes Bord N 908720 T LUCIE 92332829</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>229000</v>
+        <v>0</v>
       </c>
       <c r="F42" t="n">
-        <v>0</v>
+        <v>2309475</v>
       </c>
       <c r="G42" t="n">
-        <v>5284397</v>
+        <v>346007449</v>
       </c>
     </row>
     <row r="43">
@@ -1660,27 +1660,27 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>18/11/2025</t>
+          <t>19/11/2025</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>18/11/2025</t>
+          <t>21/11/2025</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000785 Ret cheq N 6000785 du 18/11/2025 Porteur : AGBODEKA KODJOVI</t>
+          <t>CHEQUES AUTRE BANQUE - BTCI AGBANLEPEDOGAN AGBANLEPEDOGAN</t>
         </is>
       </c>
       <c r="E43" t="n">
-        <v>349000</v>
+        <v>0</v>
       </c>
       <c r="F43" t="n">
-        <v>0</v>
+        <v>60000</v>
       </c>
       <c r="G43" t="n">
-        <v>4935397</v>
+        <v>346067449</v>
       </c>
     </row>
     <row r="44">
@@ -1689,27 +1689,27 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>18/11/2025</t>
+          <t>19/11/2025</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>18/11/2025</t>
+          <t>21/11/2025</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000793 Ret cheq N 6000793 du 18/11/2025 Porteur : KPOMEGBE ALI 91907585</t>
+          <t>CHEQUES AUTRE BANQUE - BTCI AMADAHOME AMADAHOME</t>
         </is>
       </c>
       <c r="E44" t="n">
-        <v>277000</v>
+        <v>0</v>
       </c>
       <c r="F44" t="n">
-        <v>0</v>
+        <v>588400</v>
       </c>
       <c r="G44" t="n">
-        <v>4658397</v>
+        <v>346655849</v>
       </c>
     </row>
     <row r="45">
@@ -1718,27 +1718,27 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>19/11/2025</t>
+          <t>20/11/2025</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>19/11/2025</t>
+          <t>20/11/2025</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000670 Ret cheq N 6000670 du 19/11/2025 - MAKO ESSOFA 90362152 Porteur : MAKO ESSOFA 90362152</t>
+          <t>ESPECES CPT 5689825 N 5689825 : TAYI KOKU FIAM 90595933</t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>202000</v>
+        <v>1000000</v>
       </c>
       <c r="F45" t="n">
         <v>0</v>
       </c>
       <c r="G45" t="n">
-        <v>4456397</v>
+        <v>345655849</v>
       </c>
     </row>
     <row r="46">
@@ -1757,17 +1757,17 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000782 Ret cheq N 6000782</t>
+          <t>ESPECE CPT COURANT especes Bord N 909092 T LUCIE 92332829</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>322500</v>
+        <v>0</v>
       </c>
       <c r="F46" t="n">
-        <v>0</v>
+        <v>2391700</v>
       </c>
       <c r="G46" t="n">
-        <v>4133897</v>
+        <v>348047549</v>
       </c>
     </row>
     <row r="47">
@@ -1781,22 +1781,22 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>20/11/2025</t>
+          <t>21/11/2025</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000665 Ret cheq N 6000665 du 20/11/2025 Porteur : OUENANGOU TAMA 91096960</t>
+          <t>CHEQUES SBF INTERNE chq OTG</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>51000</v>
+        <v>0</v>
       </c>
       <c r="F47" t="n">
-        <v>0</v>
+        <v>500000</v>
       </c>
       <c r="G47" t="n">
-        <v>4082897</v>
+        <v>348547549</v>
       </c>
     </row>
     <row r="48">
@@ -1805,27 +1805,27 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>21/11/2025</t>
+          <t>20/11/2025</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>21/11/2025</t>
+          <t>20/11/2025</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000798 Ret cheq N 6000798 du 21/11/2025 Porteur : N'BOUKE ESSI DELALI 90 97 97 27</t>
+          <t>FACT DU 071125</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>352500</v>
+        <v>0</v>
       </c>
       <c r="F48" t="n">
-        <v>0</v>
+        <v>182510</v>
       </c>
       <c r="G48" t="n">
-        <v>3730397</v>
+        <v>348730059</v>
       </c>
     </row>
     <row r="49">
@@ -1844,17 +1844,17 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>VERSEMENT ESPECE CPT COURANT Versement especes Bord N 909502 ATTIGLOH KOFFI MAWULI 93174711</t>
+          <t>ESPECE CPT COURANT especes Bord N 909405 T LUCIE 92332829</t>
         </is>
       </c>
       <c r="E49" t="n">
         <v>0</v>
       </c>
       <c r="F49" t="n">
-        <v>1900</v>
+        <v>2206500</v>
       </c>
       <c r="G49" t="n">
-        <v>3732297</v>
+        <v>350936559</v>
       </c>
     </row>
     <row r="50">
@@ -1863,27 +1863,27 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>24/11/2025</t>
+          <t>21/11/2025</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>24/11/2025</t>
+          <t>20/11/2025</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000660 Ret cheq N 6000660 du 24/11/2025 Porteur : DOLOU ESSOLAKINA 90242454</t>
+          <t>CHEQUES SBF INTERNE chq OTG n 5810896 191638 - 01001 -</t>
         </is>
       </c>
       <c r="E50" t="n">
-        <v>319000</v>
+        <v>78517</v>
       </c>
       <c r="F50" t="n">
         <v>0</v>
       </c>
       <c r="G50" t="n">
-        <v>3413297</v>
+        <v>350858042</v>
       </c>
     </row>
     <row r="51">
@@ -1892,27 +1892,27 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>24/11/2025</t>
+          <t>21/11/2025</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>24/11/2025</t>
+          <t>20/11/2025</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000773 Ret cheq N 6000773 du 24/11/2025 Porteur : KANTCHIRE YENDOUBE 90204049</t>
+          <t>CHEQUES SBF INTERNE chq OTG n 5810888 191639 - 01001 -</t>
         </is>
       </c>
       <c r="E51" t="n">
-        <v>349000</v>
+        <v>376881</v>
       </c>
       <c r="F51" t="n">
         <v>0</v>
       </c>
       <c r="G51" t="n">
-        <v>3064297</v>
+        <v>350481161</v>
       </c>
     </row>
     <row r="52">
@@ -1921,27 +1921,27 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>24/11/2025</t>
+          <t>21/11/2025</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>24/11/2025</t>
+          <t>20/11/2025</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000786 Ret cheq N 6000786 du 24/11/2025 Porteur : LARE SOUMBAKO 91073443</t>
+          <t>RETOUR DE COMPENSATION OTG n 5810891</t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>448000</v>
+        <v>2077045</v>
       </c>
       <c r="F52" t="n">
         <v>0</v>
       </c>
       <c r="G52" t="n">
-        <v>2616297</v>
+        <v>348404116</v>
       </c>
     </row>
     <row r="53">
@@ -1950,27 +1950,27 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>24/11/2025</t>
+          <t>21/11/2025</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>24/11/2025</t>
+          <t>20/11/2025</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000664 Ret cheq N 6000664 du 24/11/2025 Porteur : SEDJRO AFANTOLOU 93237688</t>
+          <t>RETOUR DE COMPENSATION OTG n 5810887</t>
         </is>
       </c>
       <c r="E53" t="n">
-        <v>153000</v>
+        <v>1501063</v>
       </c>
       <c r="F53" t="n">
         <v>0</v>
       </c>
       <c r="G53" t="n">
-        <v>2463297</v>
+        <v>346903053</v>
       </c>
     </row>
     <row r="54">
@@ -1979,27 +1979,27 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>25/11/2025</t>
+          <t>21/11/2025</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>25/11/2025</t>
+          <t>20/11/2025</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000661 Ret cheq N 6000661 du 25/11/2025 Porteur : BASSABI DERMANE SANDUIIRI 90716263</t>
+          <t>RETOUR DE COMPENSATION OTG n 5810892</t>
         </is>
       </c>
       <c r="E54" t="n">
-        <v>227000</v>
+        <v>1500000</v>
       </c>
       <c r="F54" t="n">
         <v>0</v>
       </c>
       <c r="G54" t="n">
-        <v>2236297</v>
+        <v>345403053</v>
       </c>
     </row>
     <row r="55">
@@ -2008,27 +2008,27 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>26/11/2025</t>
+          <t>21/11/2025</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>26/11/2025</t>
+          <t>20/11/2025</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000796 Ret cheq N 6000796</t>
+          <t>RETOUR DE COMPENSATION OTG n 5810890</t>
         </is>
       </c>
       <c r="E55" t="n">
-        <v>77000</v>
+        <v>1355960</v>
       </c>
       <c r="F55" t="n">
         <v>0</v>
       </c>
       <c r="G55" t="n">
-        <v>2159297</v>
+        <v>344047093</v>
       </c>
     </row>
     <row r="56">
@@ -2037,27 +2037,27 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>26/11/2025</t>
+          <t>21/11/2025</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>26/11/2025</t>
+          <t>20/11/2025</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>RETRAIT ESPECES CPT 6000669 Ret cheq N 6000669 du 26/11/2025 Porteur : DOMPE KODJOVI 91684229</t>
+          <t>M BR 2500029 multiple INH</t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>406000</v>
+        <v>1054505</v>
       </c>
       <c r="F56" t="n">
         <v>0</v>
       </c>
       <c r="G56" t="n">
-        <v>1753297</v>
+        <v>342992588</v>
       </c>
     </row>
     <row r="57">
@@ -2066,27 +2066,1100 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
+          <t>24/11/2025</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>24/11/2025</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>ESPECES CPT 5689526 N 5689526 : ABALO PADANAM 90156097</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>499550</v>
+      </c>
+      <c r="F57" t="n">
+        <v>0</v>
+      </c>
+      <c r="G57" t="n">
+        <v>342493038</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>24/11/2025</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>24/11/2025</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>ESPECE CPT COURANT especes Bord N 224730 91392434</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>0</v>
+      </c>
+      <c r="F58" t="n">
+        <v>115000</v>
+      </c>
+      <c r="G58" t="n">
+        <v>342608038</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>24/11/2025</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>24/11/2025</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>ESPECE CPT COURANT especes Bord N 910189 K EDEM 90978863</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>0</v>
+      </c>
+      <c r="F59" t="n">
+        <v>457475</v>
+      </c>
+      <c r="G59" t="n">
+        <v>343065513</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>24/11/2025</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>24/11/2025</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>ESPECE CPT COURANT especes Bord N 910192 K EDEM 90978863</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>0</v>
+      </c>
+      <c r="F60" t="n">
+        <v>2065275</v>
+      </c>
+      <c r="G60" t="n">
+        <v>345130788</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>24/11/2025</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>21/11/2025</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>RETOUR DE COMPENSATION OTG n 5810885</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>141700</v>
+      </c>
+      <c r="F61" t="n">
+        <v>0</v>
+      </c>
+      <c r="G61" t="n">
+        <v>344989088</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>24/11/2025</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>21/11/2025</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>RETOUR DE COMPENSATION OTG n 5810884</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>614760</v>
+      </c>
+      <c r="F62" t="n">
+        <v>0</v>
+      </c>
+      <c r="G62" t="n">
+        <v>344374328</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>24/11/2025</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>26/11/2025</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>CHEQUES AUTRE BANQUE - BIA AGENCE PRINCIPALE LOME PRINCIPALE LOME</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>0</v>
+      </c>
+      <c r="F63" t="n">
+        <v>240000</v>
+      </c>
+      <c r="G63" t="n">
+        <v>344614328</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>24/11/2025</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>26/11/2025</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>CHEQUES AUTRE BANQUE - UTB SOKODE SOKODE</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>0</v>
+      </c>
+      <c r="F64" t="n">
+        <v>58000</v>
+      </c>
+      <c r="G64" t="n">
+        <v>344672328</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>24/11/2025</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>25/11/2025</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>RECU COMPENSATION</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>0</v>
+      </c>
+      <c r="F65" t="n">
+        <v>306900</v>
+      </c>
+      <c r="G65" t="n">
+        <v>344979228</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>25/11/2025</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>25/11/2025</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>ESPECE CPT COURANT especes Bord N 910402 K EDEM 90978863</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>0</v>
+      </c>
+      <c r="F66" t="n">
+        <v>2188550</v>
+      </c>
+      <c r="G66" t="n">
+        <v>347167778</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>25/11/2025</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>24/11/2025</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>RETOUR DE COMPENSATION OTG n 5810897</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>735680</v>
+      </c>
+      <c r="F67" t="n">
+        <v>0</v>
+      </c>
+      <c r="G67" t="n">
+        <v>346432098</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>25/11/2025</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>24/11/2025</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>NOS CAISSES fav. BIO GROUPE LABO-SYSTEMES 154845 - 01101 - REGLEMENT</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>5007576</v>
+      </c>
+      <c r="F68" t="n">
+        <v>0</v>
+      </c>
+      <c r="G68" t="n">
+        <v>341424522</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>26/11/2025</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>26/11/2025</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>ESPECES CPT 5689528 N 5689528 : ANENYA KOMIVI EDEM 90978863</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="F69" t="n">
+        <v>0</v>
+      </c>
+      <c r="G69" t="n">
+        <v>339424522</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>26/11/2025</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>26/11/2025</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>ESPECE CPT COURANT especes Bord N 910922 K EDEM 90978863</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>0</v>
+      </c>
+      <c r="F70" t="n">
+        <v>2831600</v>
+      </c>
+      <c r="G70" t="n">
+        <v>342256122</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>26/11/2025</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>25/11/2025</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>RETOUR DE COMPENSATION OTG n 5810894</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>784800</v>
+      </c>
+      <c r="F71" t="n">
+        <v>0</v>
+      </c>
+      <c r="G71" t="n">
+        <v>341471322</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>26/11/2025</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>25/11/2025</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>MULTI CPT DEBIT SOCIETE multiple SALAIRE DU: 26/11/25</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>14853435</v>
+      </c>
+      <c r="F72" t="n">
+        <v>0</v>
+      </c>
+      <c r="G72" t="n">
+        <v>326617887</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
           <t>27/11/2025</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C73" t="inlineStr">
         <is>
           <t>27/11/2025</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>RETRAIT ESPECES CPT 6000792 Ret cheq N 6000792 du 27/11/2025 Porteur : KOUDJANE TAFAN97187002</t>
-        </is>
-      </c>
-      <c r="E57" t="n">
-        <v>388000</v>
-      </c>
-      <c r="F57" t="n">
-        <v>0</v>
-      </c>
-      <c r="G57" t="n">
-        <v>1365297</v>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>ESPECES CPT 5689527 N 5689527 : LOSSOU KOFFITS AKOLI 93313233</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="F73" t="n">
+        <v>0</v>
+      </c>
+      <c r="G73" t="n">
+        <v>321617887</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>27/11/2025</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>27/11/2025</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>ESPECE CPT COURANT especes Bord N 911249 K EDEM 90978863</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>0</v>
+      </c>
+      <c r="F74" t="n">
+        <v>2762875</v>
+      </c>
+      <c r="G74" t="n">
+        <v>324380762</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>27/11/2025</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>26/11/2025</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>CHEQUES SBF INTERNE chq OTG n 5810899 174304 - 01008 -</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>2580000</v>
+      </c>
+      <c r="F75" t="n">
+        <v>0</v>
+      </c>
+      <c r="G75" t="n">
+        <v>321800762</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>27/11/2025</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>26/11/2025</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>RETOUR DE COMPENSATION OTG n 5810907</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>1631775</v>
+      </c>
+      <c r="F76" t="n">
+        <v>0</v>
+      </c>
+      <c r="G76" t="n">
+        <v>320168987</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>27/11/2025</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>26/11/2025</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>RETOUR DE COMPENSATION OTG n 5810909</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>911476</v>
+      </c>
+      <c r="F77" t="n">
+        <v>0</v>
+      </c>
+      <c r="G77" t="n">
+        <v>319257511</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>27/11/2025</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>01/12/2025</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>CHEQUES AUTRE BANQUE - UTB CIRCULAIRE CIRCULAIRE</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>0</v>
+      </c>
+      <c r="F78" t="n">
+        <v>190350</v>
+      </c>
+      <c r="G78" t="n">
+        <v>319447861</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>27/11/2025</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>26/11/2025</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>AUTRES AGENCES fav. CAISSE NATIONALE DE SECURITE SOC 160688 - 01101 - REGLEMENT</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>2688333</v>
+      </c>
+      <c r="F79" t="n">
+        <v>0</v>
+      </c>
+      <c r="G79" t="n">
+        <v>316759528</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>27/11/2025</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>26/11/2025</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>AUTRES AGENCES fav. CAISSE NATIONALE DE SECURITE SOC 160689 - 01101 - RGLT AMU</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>1250388</v>
+      </c>
+      <c r="F80" t="n">
+        <v>0</v>
+      </c>
+      <c r="G80" t="n">
+        <v>315509140</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>27/11/2025</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>28/11/2025</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>NC AUTRES AGENCES ord. CAISSE NATIONALE DE SECURITE SOC - 01101 - RGLT FACTURES AMU</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>0</v>
+      </c>
+      <c r="F81" t="n">
+        <v>30696</v>
+      </c>
+      <c r="G81" t="n">
+        <v>315539836</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>27/11/2025</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>28/11/2025</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>NC AUTRES AGENCES ord. CAISSE NATIONALE DE SECURITE SOC - 01101 - RGLT FACT AMU</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>0</v>
+      </c>
+      <c r="F82" t="n">
+        <v>7013896</v>
+      </c>
+      <c r="G82" t="n">
+        <v>322553732</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>27/11/2025</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>27/11/2025</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>DIBURSING OFFICER reçu DIBURSING OFFICER</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>0</v>
+      </c>
+      <c r="F83" t="n">
+        <v>120000</v>
+      </c>
+      <c r="G83" t="n">
+        <v>322673732</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>28/11/2025</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>28/11/2025</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>DE TENUE DE COMPTE</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>3300</v>
+      </c>
+      <c r="F84" t="n">
+        <v>0</v>
+      </c>
+      <c r="G84" t="n">
+        <v>322670432</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>28/11/2025</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>28/11/2025</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>ESPECE CPT COURANT especes Bord N 224955 BELARO 90915582</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>0</v>
+      </c>
+      <c r="F85" t="n">
+        <v>216425</v>
+      </c>
+      <c r="G85" t="n">
+        <v>322886857</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>28/11/2025</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>28/11/2025</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>ESPECE CPT COURANT especes Bord N 911665 K EDEM 90978863</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>0</v>
+      </c>
+      <c r="F86" t="n">
+        <v>701900</v>
+      </c>
+      <c r="G86" t="n">
+        <v>323588757</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>28/11/2025</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>28/11/2025</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>ESPECE CPT COURANT especes Bord N 911667 K EDEM 90978863</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>0</v>
+      </c>
+      <c r="F87" t="n">
+        <v>1972650</v>
+      </c>
+      <c r="G87" t="n">
+        <v>325561407</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>28/11/2025</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>27/11/2025</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>RETOUR DE COMPENSATION OTG n 5810898</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>2253159</v>
+      </c>
+      <c r="F88" t="n">
+        <v>0</v>
+      </c>
+      <c r="G88" t="n">
+        <v>323308248</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>28/11/2025</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>27/11/2025</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>RETOUR DE COMPENSATION OTG n 5810906</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>359436</v>
+      </c>
+      <c r="F89" t="n">
+        <v>0</v>
+      </c>
+      <c r="G89" t="n">
+        <v>322948812</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>28/11/2025</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>27/11/2025</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>RETOUR DE COMPENSATION OTG n 5810905</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>3764729</v>
+      </c>
+      <c r="F90" t="n">
+        <v>0</v>
+      </c>
+      <c r="G90" t="n">
+        <v>319184083</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>28/11/2025</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>27/11/2025</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>RETOUR DE COMPENSATION OTG n 5810904</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>319000</v>
+      </c>
+      <c r="F91" t="n">
+        <v>0</v>
+      </c>
+      <c r="G91" t="n">
+        <v>318865083</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>28/11/2025</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>02/12/2025</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>CHEQUES AUTRE BANQUE - ECOBANK VICTOIRE VICTOIRE</t>
+        </is>
+      </c>
+      <c r="E92" t="n">
+        <v>0</v>
+      </c>
+      <c r="F92" t="n">
+        <v>316500</v>
+      </c>
+      <c r="G92" t="n">
+        <v>319181583</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>28/11/2025</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>01/12/2025</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>RECU COMPENSATION ord. OLEA SANTE TOGO 14 SANTE 251127118T</t>
+        </is>
+      </c>
+      <c r="E93" t="n">
+        <v>0</v>
+      </c>
+      <c r="F93" t="n">
+        <v>169740</v>
+      </c>
+      <c r="G93" t="n">
+        <v>319351323</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>28/11/2025</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>27/11/2025</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>DE S PRODUIT E-</t>
+        </is>
+      </c>
+      <c r="E94" t="n">
+        <v>1650</v>
+      </c>
+      <c r="F94" t="n">
+        <v>0</v>
+      </c>
+      <c r="G94" t="n">
+        <v>319349673</v>
       </c>
     </row>
   </sheetData>

</xml_diff>